<commit_message>
se agregan terminos y condiciones
</commit_message>
<xml_diff>
--- a/imagenes_guardadas/plantilla_mantenimiento.xlsx
+++ b/imagenes_guardadas/plantilla_mantenimiento.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\acrivera-sis\imagenes_guardadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23520BE0-2A78-4C82-8E71-746D470AF991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAD27BC0-A436-490E-BB72-A42E4EA014D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4A4F58DA-A499-4342-B7EA-C20A63C4C227}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{4A4F58DA-A499-4342-B7EA-C20A63C4C227}"/>
   </bookViews>
   <sheets>
     <sheet name="plantilla" sheetId="1" r:id="rId1"/>
@@ -475,6 +475,33 @@
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -484,17 +511,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -505,31 +526,10 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -992,21 +992,21 @@
       <c r="M6" s="7"/>
     </row>
     <row r="7" spans="1:13">
-      <c r="B7" s="51" t="s">
+      <c r="B7" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="51"/>
+      <c r="E7" s="51"/>
       <c r="F7" s="44"/>
-      <c r="H7" s="52" t="s">
+      <c r="H7" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="I7" s="52"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="52"/>
-      <c r="L7" s="48"/>
-      <c r="M7" s="53"/>
+      <c r="I7" s="51"/>
+      <c r="J7" s="51"/>
+      <c r="K7" s="51"/>
+      <c r="L7" s="57"/>
+      <c r="M7" s="60"/>
     </row>
     <row r="8" spans="1:13" ht="7.5" customHeight="1">
       <c r="B8" s="11"/>
@@ -1014,17 +1014,17 @@
     </row>
     <row r="9" spans="1:13" ht="13.5">
       <c r="A9" s="9"/>
-      <c r="B9" s="51" t="s">
+      <c r="B9" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="52"/>
+      <c r="C9" s="51"/>
       <c r="D9" s="45"/>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
-      <c r="H9" s="52" t="s">
+      <c r="H9" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="I9" s="52"/>
+      <c r="I9" s="51"/>
       <c r="J9" s="45"/>
       <c r="K9" s="13"/>
       <c r="L9" s="9"/>
@@ -1047,22 +1047,22 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="9"/>
-      <c r="B11" s="51" t="s">
+      <c r="B11" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="52"/>
+      <c r="C11" s="51"/>
       <c r="D11" s="9"/>
-      <c r="E11" s="48" t="s">
+      <c r="E11" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="F11" s="48"/>
-      <c r="G11" s="48"/>
-      <c r="H11" s="48"/>
-      <c r="I11" s="48"/>
-      <c r="J11" s="48"/>
-      <c r="K11" s="48"/>
-      <c r="L11" s="48"/>
-      <c r="M11" s="53"/>
+      <c r="F11" s="57"/>
+      <c r="G11" s="57"/>
+      <c r="H11" s="57"/>
+      <c r="I11" s="57"/>
+      <c r="J11" s="57"/>
+      <c r="K11" s="57"/>
+      <c r="L11" s="57"/>
+      <c r="M11" s="60"/>
     </row>
     <row r="12" spans="1:13" ht="7.5" customHeight="1" thickBot="1">
       <c r="A12" s="9"/>
@@ -1110,20 +1110,20 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="9"/>
-      <c r="B15" s="46" t="s">
+      <c r="B15" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="47"/>
+      <c r="C15" s="56"/>
       <c r="D15" s="21"/>
       <c r="E15" s="9"/>
-      <c r="F15" s="48"/>
-      <c r="G15" s="48"/>
-      <c r="H15" s="48"/>
-      <c r="I15" s="48"/>
-      <c r="J15" s="48"/>
-      <c r="K15" s="48"/>
-      <c r="L15" s="48"/>
-      <c r="M15" s="53"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="57"/>
+      <c r="I15" s="57"/>
+      <c r="J15" s="57"/>
+      <c r="K15" s="57"/>
+      <c r="L15" s="57"/>
+      <c r="M15" s="60"/>
     </row>
     <row r="16" spans="1:13" ht="7.5" customHeight="1">
       <c r="B16" s="11"/>
@@ -1133,18 +1133,18 @@
       <c r="B17" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="48"/>
-      <c r="D17" s="48"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="48"/>
-      <c r="H17" s="47" t="s">
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="57"/>
+      <c r="H17" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="I17" s="47"/>
-      <c r="J17" s="54"/>
-      <c r="K17" s="54"/>
-      <c r="L17" s="54"/>
-      <c r="M17" s="55"/>
+      <c r="I17" s="56"/>
+      <c r="J17" s="61"/>
+      <c r="K17" s="61"/>
+      <c r="L17" s="61"/>
+      <c r="M17" s="62"/>
     </row>
     <row r="18" spans="1:13" ht="7.5" customHeight="1">
       <c r="B18" s="11"/>
@@ -1152,21 +1152,21 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="9"/>
-      <c r="B19" s="46" t="s">
+      <c r="B19" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="47"/>
-      <c r="D19" s="48"/>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
-      <c r="H19" s="47" t="s">
+      <c r="C19" s="56"/>
+      <c r="D19" s="57"/>
+      <c r="E19" s="57"/>
+      <c r="F19" s="57"/>
+      <c r="H19" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="I19" s="47"/>
-      <c r="J19" s="49"/>
-      <c r="K19" s="49"/>
-      <c r="L19" s="49"/>
-      <c r="M19" s="50"/>
+      <c r="I19" s="56"/>
+      <c r="J19" s="48"/>
+      <c r="K19" s="48"/>
+      <c r="L19" s="48"/>
+      <c r="M19" s="49"/>
     </row>
     <row r="20" spans="1:13" ht="7.5" customHeight="1">
       <c r="B20" s="11"/>
@@ -1174,21 +1174,21 @@
     </row>
     <row r="21" spans="1:13">
       <c r="A21" s="9"/>
-      <c r="B21" s="46" t="s">
+      <c r="B21" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="47"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
+      <c r="C21" s="56"/>
+      <c r="D21" s="57"/>
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
       <c r="H21" s="21" t="s">
         <v>14</v>
       </c>
       <c r="I21" s="21"/>
-      <c r="J21" s="49"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="49"/>
-      <c r="M21" s="50"/>
+      <c r="J21" s="48"/>
+      <c r="K21" s="48"/>
+      <c r="L21" s="48"/>
+      <c r="M21" s="49"/>
     </row>
     <row r="22" spans="1:13" ht="7.5" customHeight="1">
       <c r="B22" s="11"/>
@@ -1196,22 +1196,22 @@
     </row>
     <row r="23" spans="1:13">
       <c r="A23" s="9"/>
-      <c r="B23" s="51" t="s">
+      <c r="B23" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="C23" s="52"/>
+      <c r="C23" s="51"/>
       <c r="D23" s="9"/>
-      <c r="E23" s="49" t="s">
+      <c r="E23" s="48" t="s">
         <v>15</v>
       </c>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="49"/>
-      <c r="K23" s="49"/>
-      <c r="L23" s="49"/>
-      <c r="M23" s="50"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="48"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
+      <c r="K23" s="48"/>
+      <c r="L23" s="48"/>
+      <c r="M23" s="49"/>
     </row>
     <row r="24" spans="1:13" ht="7.5" customHeight="1" thickBot="1">
       <c r="A24" s="9"/>
@@ -1251,21 +1251,21 @@
       <c r="M26" s="7"/>
     </row>
     <row r="27" spans="1:13">
-      <c r="B27" s="56" t="s">
+      <c r="B27" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="C27" s="57"/>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="57"/>
-      <c r="H27" s="57" t="s">
+      <c r="C27" s="46"/>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="46"/>
+      <c r="H27" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="I27" s="57"/>
-      <c r="J27" s="57"/>
-      <c r="K27" s="57"/>
-      <c r="L27" s="57"/>
-      <c r="M27" s="58"/>
+      <c r="I27" s="46"/>
+      <c r="J27" s="46"/>
+      <c r="K27" s="46"/>
+      <c r="L27" s="46"/>
+      <c r="M27" s="47"/>
     </row>
     <row r="28" spans="1:13" ht="7.5" customHeight="1">
       <c r="A28" s="9"/>
@@ -1277,22 +1277,22 @@
     </row>
     <row r="29" spans="1:13" ht="13.5">
       <c r="A29" s="9"/>
-      <c r="B29" s="51" t="s">
+      <c r="B29" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="52"/>
+      <c r="C29" s="51"/>
       <c r="D29" s="9"/>
       <c r="E29" s="13"/>
       <c r="F29" s="9"/>
-      <c r="G29" s="52" t="s">
+      <c r="G29" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="H29" s="52"/>
-      <c r="I29" s="52"/>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
       <c r="J29" s="9"/>
       <c r="K29" s="13"/>
       <c r="L29" s="13"/>
-      <c r="M29" s="59"/>
+      <c r="M29" s="58"/>
     </row>
     <row r="30" spans="1:13" ht="7.5" customHeight="1">
       <c r="B30" s="28"/>
@@ -1303,26 +1303,26 @@
       <c r="J30" s="9"/>
       <c r="K30" s="9"/>
       <c r="L30" s="9"/>
-      <c r="M30" s="60"/>
+      <c r="M30" s="59"/>
     </row>
     <row r="31" spans="1:13" ht="13.5">
       <c r="A31" s="9"/>
-      <c r="B31" s="51" t="s">
+      <c r="B31" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="C31" s="52"/>
+      <c r="C31" s="51"/>
       <c r="D31" s="9"/>
       <c r="E31" s="13"/>
       <c r="F31" s="9"/>
-      <c r="G31" s="52" t="s">
+      <c r="G31" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="H31" s="52"/>
-      <c r="I31" s="52"/>
+      <c r="H31" s="51"/>
+      <c r="I31" s="51"/>
       <c r="J31" s="9"/>
       <c r="K31" s="13"/>
       <c r="L31" s="13"/>
-      <c r="M31" s="60"/>
+      <c r="M31" s="59"/>
     </row>
     <row r="32" spans="1:13" ht="7.5" customHeight="1">
       <c r="B32" s="8"/>
@@ -1337,18 +1337,18 @@
     </row>
     <row r="33" spans="1:13" ht="13.5">
       <c r="A33" s="9"/>
-      <c r="B33" s="51" t="s">
+      <c r="B33" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="C33" s="52"/>
+      <c r="C33" s="51"/>
       <c r="D33" s="9"/>
       <c r="E33" s="13"/>
       <c r="F33" s="9"/>
-      <c r="G33" s="52" t="s">
+      <c r="G33" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="H33" s="52"/>
-      <c r="I33" s="52"/>
+      <c r="H33" s="51"/>
+      <c r="I33" s="51"/>
       <c r="J33" s="9"/>
       <c r="K33" s="29"/>
       <c r="L33" s="9"/>
@@ -1367,17 +1367,17 @@
     </row>
     <row r="35" spans="1:13" ht="13.5">
       <c r="A35" s="9"/>
-      <c r="B35" s="51" t="s">
+      <c r="B35" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="C35" s="52"/>
+      <c r="C35" s="51"/>
       <c r="D35" s="9"/>
       <c r="E35" s="13"/>
-      <c r="G35" s="52" t="s">
+      <c r="G35" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="H35" s="52"/>
-      <c r="I35" s="52"/>
+      <c r="H35" s="51"/>
+      <c r="I35" s="51"/>
       <c r="J35" s="9"/>
       <c r="K35" s="29"/>
       <c r="L35" s="9"/>
@@ -1396,18 +1396,18 @@
     </row>
     <row r="37" spans="1:13" ht="13.5">
       <c r="A37" s="9"/>
-      <c r="B37" s="51" t="s">
+      <c r="B37" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="C37" s="52"/>
+      <c r="C37" s="51"/>
       <c r="D37" s="9"/>
       <c r="E37" s="13"/>
       <c r="F37" s="18"/>
-      <c r="G37" s="52" t="s">
+      <c r="G37" s="51" t="s">
         <v>27</v>
       </c>
-      <c r="H37" s="52"/>
-      <c r="I37" s="52"/>
+      <c r="H37" s="51"/>
+      <c r="I37" s="51"/>
       <c r="J37" s="9"/>
       <c r="K37" s="29"/>
       <c r="L37" s="18"/>
@@ -1749,27 +1749,27 @@
     </row>
     <row r="73" spans="1:13">
       <c r="A73" s="18"/>
-      <c r="B73" s="56" t="s">
+      <c r="B73" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="C73" s="57"/>
+      <c r="C73" s="46"/>
       <c r="D73" s="18"/>
       <c r="E73" s="18"/>
-      <c r="F73" s="57" t="s">
+      <c r="F73" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="G73" s="57"/>
-      <c r="H73" s="57"/>
-      <c r="I73" s="57"/>
-      <c r="L73" s="57" t="s">
+      <c r="G73" s="46"/>
+      <c r="H73" s="46"/>
+      <c r="I73" s="46"/>
+      <c r="L73" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="M73" s="58"/>
+      <c r="M73" s="47"/>
     </row>
     <row r="74" spans="1:13">
       <c r="A74" s="18"/>
-      <c r="B74" s="63"/>
-      <c r="C74" s="64"/>
+      <c r="B74" s="53"/>
+      <c r="C74" s="54"/>
       <c r="D74" s="18"/>
       <c r="E74" s="18"/>
       <c r="F74" s="18"/>
@@ -1786,18 +1786,18 @@
     </row>
     <row r="76" spans="1:13" ht="33" customHeight="1">
       <c r="A76" s="18"/>
-      <c r="B76" s="61"/>
-      <c r="C76" s="62"/>
+      <c r="B76" s="63"/>
+      <c r="C76" s="64"/>
       <c r="D76" s="18"/>
       <c r="E76" s="18"/>
-      <c r="F76" s="49"/>
-      <c r="G76" s="49"/>
-      <c r="H76" s="49"/>
-      <c r="I76" s="49"/>
-      <c r="L76" s="49" t="s">
+      <c r="F76" s="48"/>
+      <c r="G76" s="48"/>
+      <c r="H76" s="48"/>
+      <c r="I76" s="48"/>
+      <c r="L76" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="M76" s="50"/>
+      <c r="M76" s="49"/>
     </row>
     <row r="77" spans="1:13" ht="8.25" customHeight="1" thickBot="1">
       <c r="B77" s="34"/>
@@ -1819,31 +1819,6 @@
     <row r="79" spans="1:13" ht="15.75" hidden="1" customHeight="1"/>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="L73:M73"/>
-    <mergeCell ref="F76:I76"/>
-    <mergeCell ref="L76:M76"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="F73:I73"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="J21:M21"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="E23:M23"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="H27:M27"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="M29:M31"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="G31:I31"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="H19:I19"/>
@@ -1860,6 +1835,31 @@
     <mergeCell ref="C17:F17"/>
     <mergeCell ref="H17:I17"/>
     <mergeCell ref="J17:M17"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="J21:M21"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="E23:M23"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="H27:M27"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="M29:M31"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="L73:M73"/>
+    <mergeCell ref="F76:I76"/>
+    <mergeCell ref="L76:M76"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="F73:I73"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B74:C74"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0" bottom="0" header="0" footer="0.19685039370078741"/>

</xml_diff>